<commit_message>
Enrich Excel seed data: 7 geometries, 10 candidates, 7 observations, 4 product ideas, 4 sources; agents generate 10 concepts
</commit_message>
<xml_diff>
--- a/data/geomolecular_template.xlsx
+++ b/data/geomolecular_template.xlsx
@@ -140,8 +140,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BiologicalDefinitionsTable" displayName="BiologicalDefinitionsTable" ref="A1:G3" headerRowCount="1">
-  <autoFilter ref="A1:G3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BiologicalDefinitionsTable" displayName="BiologicalDefinitionsTable" ref="A1:G7" headerRowCount="1">
+  <autoFilter ref="A1:G7"/>
   <tableColumns count="7">
     <tableColumn id="1" name="bio_id"/>
     <tableColumn id="2" name="term"/>
@@ -156,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GeometrySignaturesTable" displayName="GeometrySignaturesTable" ref="A1:K3" headerRowCount="1">
-  <autoFilter ref="A1:K3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GeometrySignaturesTable" displayName="GeometrySignaturesTable" ref="A1:K8" headerRowCount="1">
+  <autoFilter ref="A1:K8"/>
   <tableColumns count="11">
     <tableColumn id="1" name="geometry_id"/>
     <tableColumn id="2" name="geometry_name"/>
@@ -176,8 +176,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CandidateMaterialsTable" displayName="CandidateMaterialsTable" ref="A1:H3" headerRowCount="1">
-  <autoFilter ref="A1:H3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CandidateMaterialsTable" displayName="CandidateMaterialsTable" ref="A1:H11" headerRowCount="1">
+  <autoFilter ref="A1:H11"/>
   <tableColumns count="8">
     <tableColumn id="1" name="candidate_id"/>
     <tableColumn id="2" name="name"/>
@@ -193,8 +193,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ObservationsTable" displayName="ObservationsTable" ref="A1:I2" headerRowCount="1">
-  <autoFilter ref="A1:I2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ObservationsTable" displayName="ObservationsTable" ref="A1:I8" headerRowCount="1">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="observation_id"/>
     <tableColumn id="2" name="candidate_id"/>
@@ -211,8 +211,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:F2" headerRowCount="1">
-  <autoFilter ref="A1:F2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:F5" headerRowCount="1">
+  <autoFilter ref="A1:F5"/>
   <tableColumns count="6">
     <tableColumn id="1" name="source_id"/>
     <tableColumn id="2" name="title"/>
@@ -226,8 +226,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProductIdeasTable" displayName="ProductIdeasTable" ref="A1:H2" headerRowCount="1">
-  <autoFilter ref="A1:H2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ProductIdeasTable" displayName="ProductIdeasTable" ref="A1:H5" headerRowCount="1">
+  <autoFilter ref="A1:H5"/>
   <tableColumns count="8">
     <tableColumn id="1" name="idea_id"/>
     <tableColumn id="2" name="title"/>
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -651,6 +651,154 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>SRC-PROJECT-NOTE-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BIO-SURFACE-ADHESION-REPEL</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Surface adhesion repulsion</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>behavior</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Organism avoids or cannot maintain contact with a treated surface.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Confirms whether a geometry-linked surface film or interface pattern changes contact behavior.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Do not infer pesticidal or medical surface treatment efficacy.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SRC-PROJECT-NOTE-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BIO-MOSQUITO-ATTRACTION</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mosquito attraction</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>behavior</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Movement of mosquitoes toward a carbon dioxide or skin-emission mimic.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Confirms whether a geometry-linked breath-mimic or skin-odor plume attracts mosquitoes.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Do not infer repellency inverse without separate validation.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BIO-RECEPTOR-POCKET-FIT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Receptor pocket geometric fit</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pharmacology-proxy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Hypothetical binding based on complementary shape and polarity between molecule and receptor cavity.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Confirms whether a geometry-linked molecular shape could theoretically fit a known receptor pocket.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>This is geometric hypothesis only; no pharmacological claim or dosing is implied.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BIO-SKIN-BARRIER-PASSAGE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Skin barrier passage geometry</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dermatology-proxy</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Observed or hypothesized permeation through stratum corneum lipid matrix.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Confirms whether a geometry-linked amphiphilic or small-polar pattern could traverse skin layers.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>No medical delivery claim without permeation measurement and safety review.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
         </is>
       </c>
     </row>
@@ -668,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -801,57 +949,342 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>GEO-VOLATILE-PLUME-PULSE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Volatile plume temporal pulse</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Volatile Plumes</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>waveform</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>pulsed release nodes</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>room to organism</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>polarity oscillation</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>intermittent release</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Odor releases in bursts rather than steady stream; temporal pattern may trigger different behavior than constant exposure.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Behavior identical between steady and pulsed release at same average concentration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>GEO-SURFACE-FILM-INTERFACE</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Surface film interface</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Surface Films</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>plane</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>asymmetric</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>two-phase interface</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>surface to organism</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>amphiphilic boundary</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>adhesive/static</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Thin film, meniscus, residue, or coating changes contact behavior at an interface.</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Effect occurs without contact or surface interaction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GEO-BINDING-POCKET-CAVITY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Binding pocket cavity</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Binding Pockets</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>cavity</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>chiral</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>enclosed pocket with channel</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>molecular</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>hydrophobic pocket with polar rim</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>static/lock-and-key</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Complementary shape and polarity distribution allow molecular docking into a receptor cavity.</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>No measurable shape complementarity or binding affinity data available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GEO-SKIN-LAMELLAR-LAYER</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Skin lamellar lipid layer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Surface Films</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>layered lattice</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>bilayer periodic</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>stacked sheets with defects</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>cellular</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>amphiphilic lamellae</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>static/diffusive</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Lipid bilayers arranged in stacked sheets; hydrophilic and hydrophobic regions alternate. Permeation depends on defect geometry and molecule aspect ratio.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No lipid bilayer structure or skin barrier model available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GEO-TEMPORAL-PULSE-TRAIN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Temporal pulse train</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Temporal Pulses</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>waveform</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>discrete time series</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>time-series</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>on/off polarity</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>oscillating</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Repetitive stimulus bursts at fixed or variable intervals; entrainment or habituation may depend on frequency and duty cycle.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Continuous stimulus produces identical behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GEO-SURFACE-TEXTURE-RIDGE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Surface texture ridge</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Surface Films</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>line array</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>parallel ridges with grooves</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>surface to organism</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>hydrophobic ridge / hydrophilic groove</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>static/topographic</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Micro-ridges or grooves change wettability and contact angle; affects droplet retention or organism attachment.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Smooth surface produces identical contact behavior.</t>
         </is>
       </c>
     </row>
@@ -869,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1008,6 +1441,342 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CAND-YEAST-BLOOM-MASH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Yeast bloom mash</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-GRADIENT,GEO-VOLATILE-PLUME-PULSE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BIO-FLY-ATTRACTION,BIO-MOSQUITO-ATTRACTION</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Fermented grain mash with active yeast produces intermittent CO2 and volatile bursts. Geometry combines steady plume and temporal pulse.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SRC-RECIPE-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CAND-ESSENTIAL-OIL-DIFFUSER</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Essential oil diffuser</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>household</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-PULSE</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BIO-GNAT-FLIGHT-REDUCTION</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Ultrasonic diffuser releases essential oils in intermittent bursts; temporal pulse geometry may differ from steady evaporative source.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CAND-SOAP-FILM-RESIDUE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Soap film residue</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>household</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>GEO-SURFACE-FILM-INTERFACE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BIO-SURFACE-ADHESION-REPEL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Thin soap film left on surface changes contact angle and may reduce insect landing or adhesion.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CAND-CITRONELLA-CANDLE</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Citronella candle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>household</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-GRADIENT,GEO-TEMPORAL-PULSE-TRAIN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BIO-MOSQUITO-ATTRACTION,BIO-GNAT-FLIGHT-REDUCTION</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Burning candle produces steady volatile gradient and periodic heat-driven convection pulses. Geometry is compound.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CAND-CAPSAICIN-EXTRACT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Capsaicin extract</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>botanical</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>GEO-BINDING-POCKET-CAVITY</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BIO-RECEPTOR-POCKET-FIT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Capsaicin has a vanillyl group and hydrophobic tail that may fit TRPV1 receptor pocket geometry.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CAND-MENTHOL-CRYSTAL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Menthol crystal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>botanical</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GEO-BINDING-POCKET-CAVITY,GEO-SKIN-LAMELLAR-LAYER</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BIO-RECEPTOR-POCKET-FIT,BIO-SKIN-BARRIER-PASSAGE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Menthol is small, amphiphilic, and has a cyclohexanol ring that may fit TRPM8 geometry while traversing skin lipid lamellae.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CAND-ALOE-VERA-GEL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Aloe vera gel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>botanical</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GEO-SKIN-LAMELLAR-LAYER</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BIO-SKIN-BARRIER-PASSAGE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Polysaccharide gel may create a surface film that alters skin barrier geometry and moisture retention.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>needs review</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CAND-BAKING-SODA-PASTE</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Baking soda paste</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>household</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GEO-SURFACE-TEXTURE-RIDGE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BIO-SURFACE-ADHESION-REPEL</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Powder-in-water paste dries to a micro-ridged residue that may alter surface contact geometry.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>low concern</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1022,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1130,6 +1899,288 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OBS-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CAND-YEAST-BLOOM-MASH</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-PULSE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>BIO-MOSQUITO-ATTRACTION</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Backyard fermentation experiment</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mosquitoes appeared in waves correlated with visible CO2 bubble bursts from the mash.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>No trap or counterfactual; may be attracted to heat, moisture, or other cues.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SRC-RECIPE-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OBS-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CAND-ESSENTIAL-OIL-DIFFUSER</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-PULSE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BIO-GNAT-FLIGHT-REDUCTION</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Kitchen counter observation</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Gnat presence near fruit bowl reduced when diffuser was active on intermittent mode; steady mode had weaker apparent effect.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>No blinded or replicated trial; humidity change confounder.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OBS-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CAND-SOAP-FILM-RESIDUE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GEO-SURFACE-FILM-INTERFACE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BIO-SURFACE-ADHESION-REPEL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bathroom mirror cleaning test</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Flies appeared to avoid landing on mirror surface with visible soap streaks compared to untreated mirror.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Mirror reflection confounder; no controlled surface pair.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OBS-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CAND-MENTHOL-CRYSTAL</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GEO-BINDING-POCKET-CAVITY</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BIO-RECEPTOR-POCKET-FIT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Literature-derived hypothesis</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Menthol cyclohexanol ring size and hydroxyl position match known TRPM8 pocket geometry in docking models.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>In silico only; no wet-lab binding assay.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OBS-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CAND-MENTHOL-CRYSTAL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GEO-SKIN-LAMELLAR-LAYER</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BIO-SKIN-BARRIER-PASSAGE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Transdermal patch literature review</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Menthol enhances permeation of co-applied compounds through stratum corneum; may create defects in lipid lamellae.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Mechanism not fully resolved; may also act via keratinocyte disruption.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OBS-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CAND-CITRONELLA-CANDLE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GEO-TEMPORAL-PULSE-TRAIN</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BIO-GNAT-FLIGHT-REDUCTION</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Patio evening observation</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Gnat annoyance seemed lower near lit citronella candle than near unlit candle of same size and shape.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Heat, light, and convection confounders; no chemical-only control.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1144,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1216,6 +2267,102 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Seed source used to demonstrate schema only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SRC-HOUSEHOLD-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Household observation collection</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>observation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>anecdotal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Anecdotal household notes collected during informal observation periods.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SRC-MEDICAL-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Medical pharmacology hypothesis notes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>hypothesis</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Hypothesis notes for geometric docking and dermal passage; not clinical evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SRC-RECIPE-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fermentation recipe observation log</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>recipe</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>local</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>anecdotal</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Observations made during home fermentation experiments; not controlled.</t>
         </is>
       </c>
     </row>
@@ -1233,7 +2380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1330,6 +2477,132 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>IDEA-PULSE-MODULATED-AROMA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pulse modulated aroma delivery</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GEO-VOLATILE-PLUME-PULSE,GEO-TEMPORAL-PULSE-TRAIN</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CAND-ESSENTIAL-OIL-DIFFUSER,CAND-YEAST-BLOOM-MASH,CAND-CITRONELLA-CANDLE</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>household research</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Investigate whether intermittent volatile release produces different behavioral outcomes than steady release for the same total emitted mass.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Controlled observation with matched total volatile output; temporal pattern as independent variable.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Do not claim repellency, medical effect, or guaranteed behavioral change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>IDEA-GEOMETRY-LED-SURFACE-COATING</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Geometry-led surface coating screen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GEO-SURFACE-FILM-INTERFACE,GEO-SURFACE-TEXTURE-RIDGE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CAND-SOAP-FILM-RESIDUE,CAND-BAKING-SODA-PASTE</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>material science</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Compare surface residues and dried films by contact-angle geometry and micro-topography before testing biological adhesion.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Surface profilometry, contact angle measurement, biological adhesion assay, safety review.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Do not claim pesticidal, medical, or antimicrobial surface action without validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>IDEA-DERMAL-GEOMETRY-SCREEN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Dermal permeation geometry screen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GEO-SKIN-LAMELLAR-LAYER,GEO-BINDING-POCKET-CAVITY</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CAND-MENTHOL-CRYSTAL,CAND-ALOE-VERA-GEL,CAND-CAPSAICIN-EXTRACT</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>medical research</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Compare botanical candidates by skin-barrier passage geometry and receptor-pocket fit geometry before any pharmacological interpretation.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Franz cell permeation assay, receptor binding assay, safety and irritation review.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Do not claim therapeutic effect, dosing, or clinical efficacy.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add Quantum Harmonic Geometry Agent and Captain Connectivity Agent for world-changing geomolecular inference
- Implemented quantum_harmonic_geometry_agent.py with harmonic resonance simulation
- Added captain_connectivity_.py for agent connectivity monitoring
- Updated AGENTS.md with new agent roles
- Added tiktoken to requirements.txt
- Generated reports for all agents
- Enhanced Sky Net integration with quantum capabilities
</commit_message>
<xml_diff>
--- a/data/geomolecular_template.xlsx
+++ b/data/geomolecular_template.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductIdeas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExternalAgents" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShadowAgents" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -211,8 +213,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:F5" headerRowCount="1">
-  <autoFilter ref="A1:F5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A1:F10" headerRowCount="1">
+  <autoFilter ref="A1:F10"/>
   <tableColumns count="6">
     <tableColumn id="1" name="source_id"/>
     <tableColumn id="2" name="title"/>
@@ -237,6 +239,47 @@
     <tableColumn id="6" name="concept_note"/>
     <tableColumn id="7" name="required_validation"/>
     <tableColumn id="8" name="blocked_claims"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ExternalAgentsTable" displayName="ExternalAgentsTable" ref="A1:L4" headerRowCount="1">
+  <autoFilter ref="A1:L4"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="agent_id"/>
+    <tableColumn id="2" name="agent_name"/>
+    <tableColumn id="3" name="agent_type"/>
+    <tableColumn id="4" name="repository_url"/>
+    <tableColumn id="5" name="primary_function"/>
+    <tableColumn id="6" name="corpus_description"/>
+    <tableColumn id="7" name="inference_method"/>
+    <tableColumn id="8" name="action_outputs"/>
+    <tableColumn id="9" name="shadow_agent_id"/>
+    <tableColumn id="10" name="geometry_mappings"/>
+    <tableColumn id="11" name="candidate_links"/>
+    <tableColumn id="12" name="source_ids"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ShadowAgentsTable" displayName="ShadowAgentsTable" ref="A1:K4" headerRowCount="1">
+  <autoFilter ref="A1:K4"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="shadow_agent_id"/>
+    <tableColumn id="2" name="primary_agent_id"/>
+    <tableColumn id="3" name="shadow_role"/>
+    <tableColumn id="4" name="latent_dimensions"/>
+    <tableColumn id="5" name="hidden_parameters"/>
+    <tableColumn id="6" name="inference_methods"/>
+    <tableColumn id="7" name="activation_conditions"/>
+    <tableColumn id="8" name="belief_state_format"/>
+    <tableColumn id="9" name="temporal_operators"/>
+    <tableColumn id="10" name="shadow_correlations"/>
+    <tableColumn id="11" name="geometry_transitions"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2195,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2363,6 +2406,166 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Observations made during home fermentation experiments; not controlled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SRC-ALPHAFOLD-DB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AlphaFold Structure Database (EBI)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>external-api</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://alphafold.ebi.ac.uk</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Open source structure predictions for 200M+ proteins. pLDDT confidence scores provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SRC-LENIA-MATH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Lenia Mathematical Life Forms</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>simulation-framework</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://github.com/Chakazul/Lenia</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Continuous cellular automata for emergent geometry generation. Mathematical patterns not literal biology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SRC-TURING-SIM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Turing Patterns Reaction-Diffusion Simulator</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>simulation-framework</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://github.com/joserenter1a/turing_patterns</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Gray-Scott and FitzHugh-Nagumo reaction-diffusion pattern generators. Morphogenesis simulation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SRC-TURING-1952</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Turing 1952 - Chemical Basis of Morphogenesis</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1098/rstb.1952.0012</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Foundational paper on reaction-diffusion pattern formation. Philosophical Transactions Royal Society.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SRC-ALPHAFOLD-NATURE-2021</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AlphaFold Nature Paper 2021</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>paper</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41586-021-03819-2</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Highly accurate protein structure prediction with AlphaFold. CASP14 breakthrough paper.</t>
         </is>
       </c>
     </row>
@@ -2609,4 +2812,541 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>agent_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>agent_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>agent_type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>repository_url</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>primary_function</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>corpus_description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>inference_method</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>action_outputs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>shadow_agent_id</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>geometry_mappings</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>candidate_links</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>source_ids</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AGENT-ALPHAFOLD-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AlphaFold Agent</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>external-structure-predictor</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://github.com/google-deepmind/alphafold</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Structure prediction for protein geometry inference; cracks 1D sequence → 3D geometry code</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AlphaFold DB (200M+ structures), EBI API, pLDDT confidence scores</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>sequence→structure→pocket extraction→geometry mapping</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Generate geometry signatures, confidence scoring, candidate docking validation</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SHADOW-ALPHAFOLD-001</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Backbone→curve/fold, Pocket→GEO-BINDING-POCKET-CAVITY, Surface→polarity_pattern</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CAND-MENTHOL-CRYSTAL,CAND-CAPSAICIN-EXTRACT</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SRC-ALPHAFOLD-DB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGENT-LENIA-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lenia Agent</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>emergent-geometry-simulator</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://github.com/Chakazul/Lenia</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Mathematical life simulation for emergent geometry discovery; cracks geometry → life-like behavior</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Lenia pattern library (gliders, oscillators, static forms), continuous cellular automata</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>kernel params → emergent morphology → geometry classification</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Generate novel geometry signatures, model temporal dynamics, simulate autonomous patterns</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SHADOW-LENIA-001</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Glider→waveform+periodic, Oscillator→GEO-TEMPORAL-PULSE-TRAIN, Static→surface_film</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>CAND-YEAST-BLOOM-MASH,CAND-ESSENTIAL-OIL-DIFFUSER,CAND-CITRONELLA-CANDLE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SRC-LENIA-MATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGENT-TURING-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Turing Patterns Agent</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>reaction-diffusion-simulator</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://github.com/joserenter1a/turing_patterns</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Reaction-diffusion pattern generator for morphogenesis geometry; cracks chemistry → pattern → biology</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pattern library (spots, stripes, spirals, labyrinths), Gray-Scott/FitzHugh-Nagumo systems</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>RD parameters → pattern class → geometry signature (TURING-CORAL-001, etc.)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Generate morphogenesis patterns, validate temporal geometry algebra, predict bifurcations</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SHADOW-TURING-001</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Spots→periodic_point_set, Stripes→parallel_line_array, Spirals→GEO-TEMPORAL-PULSE-TRAIN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>CAND-YEAST-BLOOM-MASH,CAND-BAKING-SODA-PASTE,CAND-ESSENTIAL-OIL-DIFFUSER</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SRC-TURING-SIM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>shadow_agent_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>primary_agent_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>shadow_role</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latent_dimensions</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>hidden_parameters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>inference_methods</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>activation_conditions</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>belief_state_format</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>temporal_operators</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>shadow_correlations</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>geometry_transitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SHADOW-ALPHAFOLD-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AGENT-ALPHAFOLD-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Track latent variables in protein structure prediction (MSA entropy, attention patterns, recycling convergence)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MSA_Entropy, Attention_Pattern, Template_Weight, Recycling_Convergence</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>pLDDT_variance, MSA_depth, Convergence_RMSD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Attention rollout, Gradient-based attribution, Ensemble variance</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pLDDT_variance&gt;0.3, MSA_depth&lt;100, No_template_hits, Recycling_oscillation</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>YAML: latent_variables, confidence_distribution, convergence_status, prediction_horizon</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>d(confidence)/dt = α·(information_gain) - β·(noise_accumulation)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Alphafold flexible region → GeometrySignature dynamics parameter</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Template_vs_DeNovo, Topology_Switch, Oligomer_State transitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SHADOW-LENIA-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AGENT-LENIA-001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Track continuous state variables in mathematical life (potential field, growth kernel, stability margin)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Potential_Field, Growth_Kernel, Growth_Function, Stability_Margin</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Kernel_radius_R, Time_scale_T, Growth_center_mu, Growth_width_sigma</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Potential field interpolation, Kernel deconvolution, Stability analysis (Jacobian eigenvalues), Correlation tracking</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Period_doubling, Glider_velocity_variation&gt;5%, Pattern_emergence, Collision_imminent</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>YAML: latent_fields, geometry_parameters, pattern_tracking, stability_analysis</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>d(u)/dt = G(K * u), ∇²u, ∫u dt</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>LENIA-OSCILLATOR-001 ↔ GEO-TEMPORAL-PULSE-TRAIN (mathematical oscillator → biological pulse)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Glider→Oscillator (velocity→0), Static→Moving, Stable→Chaotic, Birth_event</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SHADOW-TURING-001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AGENT-TURING-001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Track reaction-diffusion dynamics (activator/inhibitor fields, instability growth, wavelength selection)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Activator_Field_u, Inhibitor_Field_v, Diffusion_Ratio, Reaction_Rates, Turing_Eigenvalue</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Du, Dv, f_feed_rate, k_kill_rate, λ_critical</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Spatial FFT, Phase field tracking, Defect detection, Parameter estimation</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>|∂u/∂t|&gt;threshold, Du/Dv crosses 0.5, f/k drift&gt;10%, Wavelength change&gt;20%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>YAML: latent_fields, RD_parameters, stability_analysis, pattern_metrics, temporal_evolution</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>∂u/∂t = Du·∇²u + R(u,v), ∇²u, FFT(u), ∫(u+v)dA</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>TURING-CORAL-001 ↔ GEO-SURFACE-TEXTURE-RIDGE (RD coral → surface ridge microstructure)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Homogeneous→Pattern (Turing threshold), Spots→Stripes, Stationary→Traveling, Ordered→Chaotic</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>